<commit_message>
Nieuw: risicoanalyse ISO 27001; verplichte documenten ISO 27001 bijgewerkt (37 punten)
</commit_message>
<xml_diff>
--- a/verplichte-documenten-iso-27001/maasiso-verplichte-documenten-iso-27001.xlsx
+++ b/verplichte-documenten-iso-27001/maasiso-verplichte-documenten-iso-27001.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="193">
   <si>
     <t>ISO 27001 · GRATIS SJABLOON</t>
   </si>
@@ -24,7 +24,7 @@
     <t>Verplichte documenten ISO 27001</t>
   </si>
   <si>
-    <t>Alle documenten en registraties die ISO/IEC 27001:2022 als gedocumenteerde informatie vraagt, in 21 controleerbare punten, met de clausule of beheersmaatregel bij elk punt. Versie 1.0, 16 oktober 2026.</t>
+    <t>Alle documenten en registraties die ISO/IEC 27001:2022 als gedocumenteerde informatie vraagt, in 37 controleerbare punten, met de clausule of beheersmaatregel bij elk punt. Versie 1.1, 16 oktober 2026.</t>
   </si>
   <si>
     <t>ZO GEBRUIKT U DEZE CHECKLIST</t>
@@ -51,10 +51,10 @@
     <t>KANT-EN-KLAAR</t>
   </si>
   <si>
-    <t>21 van de 21 eisen</t>
-  </si>
-  <si>
-    <t>Voor 21 van de 21 eisen staat in de laatste kolom welk document uit de ISO 27001 Toolkit die eis invult (46 documenten in Word en Excel, met implementatiegids en ingevuld voorbeeld). Zo hoeft u een ontbrekend beleid of een ontbrekende procedure niet zelf te schrijven.</t>
+    <t>37 van de 37 eisen</t>
+  </si>
+  <si>
+    <t>Voor 37 van de 37 eisen staat in de laatste kolom welk document uit de ISO 27001 Toolkit die eis invult (56 documenten in Word en Excel, met implementatiegids en ingevuld voorbeeld). Zo hoeft u een ontbrekend beleid of een ontbrekende procedure niet zelf te schrijven.</t>
   </si>
   <si>
     <t>Meer informatie</t>
@@ -99,7 +99,7 @@
     <t>maasiso.nl</t>
   </si>
   <si>
-    <t>Verplichte documenten ISO 27001 · versie 1.0 · 16 oktober 2026 · maasiso.nl</t>
+    <t>Verplichte documenten ISO 27001 · versie 1.1 · 16 oktober 2026 · maasiso.nl</t>
   </si>
   <si>
     <t>Kies in kolom D een status. In kolom I staat welk kant-en-klaar document uit de toolkit de eis invult.</t>
@@ -226,7 +226,8 @@
   </si>
   <si>
     <t xml:space="preserve">REG-001 Documentenregister
-DOC-P01 Procedure documentbeheer</t>
+DOC-P01 Procedure documentbeheer
+BWT-001 Bewaartermijnen</t>
   </si>
   <si>
     <t>V9</t>
@@ -284,6 +285,7 @@
   </si>
   <si>
     <t xml:space="preserve">AUD-P01 Procedure interne audit
+AUD-002 Auditprogramma en dekking
 T-AUD-001 Auditrapport</t>
   </si>
   <si>
@@ -296,7 +298,8 @@
     <t>9.3.3</t>
   </si>
   <si>
-    <t>DIR-P01 Procedure management review</t>
+    <t xml:space="preserve">DIR-P01 Procedure management review
+T-DIR-001 Verslag management review</t>
   </si>
   <si>
     <t>V15</t>
@@ -309,6 +312,7 @@
   </si>
   <si>
     <t xml:space="preserve">AFW-P01 Procedure afwijkingen en verbetering
+AFW-001 Register afwijkingen en verbeteringen
 T-AFW-001 Formulier afwijking en verbetering</t>
   </si>
   <si>
@@ -351,6 +355,86 @@
     <t>A4</t>
   </si>
   <si>
+    <t>Procedures om informatie te labelen volgens uw classificatieschema.</t>
+  </si>
+  <si>
+    <t>A.5.13</t>
+  </si>
+  <si>
+    <t>ISB-P06 Classificatie en uitwisseling van informatie</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>Regels, procedures of afspraken voor het overdragen van informatie, binnen de organisatie en met anderen.</t>
+  </si>
+  <si>
+    <t>A.5.14</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>Regels voor fysieke en logische toegang tot informatie en systemen.</t>
+  </si>
+  <si>
+    <t>A.5.15</t>
+  </si>
+  <si>
+    <t>ISB-P02 Toegangsbeheer</t>
+  </si>
+  <si>
+    <t>A7</t>
+  </si>
+  <si>
+    <t>Afspraken over het beheer van incidenten: processen, rollen en verantwoordelijkheden.</t>
+  </si>
+  <si>
+    <t>A.5.24</t>
+  </si>
+  <si>
+    <t>ISB-P03 Incidenten melden en afhandelen</t>
+  </si>
+  <si>
+    <t>A8</t>
+  </si>
+  <si>
+    <t>Vastgelegde procedures om op incidenten te reageren, en de registratie van incidenten.</t>
+  </si>
+  <si>
+    <t>A.5.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISB-P03 Incidenten melden en afhandelen
+INC-001 Register incidenten en datalekken</t>
+  </si>
+  <si>
+    <t>A9</t>
+  </si>
+  <si>
+    <t>Procedures voor het verzamelen en bewaren van bewijs bij incidenten.</t>
+  </si>
+  <si>
+    <t>A.5.28</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>Plannen voor continuïteit bij een verstoring, en bewijs dat ze zijn getest.</t>
+  </si>
+  <si>
+    <t>A.5.30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISB-P04 Bedrijfscontinuïteit
+T-BCT-001 Verslag test of oefening continuïteit</t>
+  </si>
+  <si>
+    <t>A11</t>
+  </si>
+  <si>
     <t>De wettelijke, regelgevende en contractuele eisen die voor informatiebeveiliging gelden, en hoe u eraan voldoet.</t>
   </si>
   <si>
@@ -360,7 +444,7 @@
     <t>REG-002 Wet- en regelgeving en contracten</t>
   </si>
   <si>
-    <t>A5</t>
+    <t>A12</t>
   </si>
   <si>
     <t>Gedocumenteerde bedieningsprocedures voor de informatieverwerkende voorzieningen.</t>
@@ -369,10 +453,32 @@
     <t>A.5.37</t>
   </si>
   <si>
-    <t>DOC-P01 Procedure documentbeheer</t>
-  </si>
-  <si>
-    <t>A6</t>
+    <t xml:space="preserve">DOC-P01 Procedure documentbeheer
+T-WIN-001 Sjabloon werkinstructie</t>
+  </si>
+  <si>
+    <t>A13</t>
+  </si>
+  <si>
+    <t>De verantwoordelijkheden voor informatiebeveiliging in de arbeidsovereenkomst.</t>
+  </si>
+  <si>
+    <t>A.6.2</t>
+  </si>
+  <si>
+    <t>HRM-P01 Procedure HR-beveiliging</t>
+  </si>
+  <si>
+    <t>A14</t>
+  </si>
+  <si>
+    <t>Een formele en bekendgemaakte disciplinaire procedure bij overtreding van het beleid.</t>
+  </si>
+  <si>
+    <t>A.6.4</t>
+  </si>
+  <si>
+    <t>A15</t>
   </si>
   <si>
     <t>Geheimhoudingsafspraken die passen bij de behoeften van de organisatie, vastgelegd en ondertekend.</t>
@@ -382,6 +488,88 @@
   </si>
   <si>
     <t>T-GHV-001 Geheimhoudingsverklaring</t>
+  </si>
+  <si>
+    <t>A16</t>
+  </si>
+  <si>
+    <t>Regels voor een opgeruimd bureau en een vergrendeld scherm.</t>
+  </si>
+  <si>
+    <t>A.7.7</t>
+  </si>
+  <si>
+    <t>A17</t>
+  </si>
+  <si>
+    <t>Vastgelegde configuraties van hardware, software, diensten en netwerken, met de beveiligingsinstellingen.</t>
+  </si>
+  <si>
+    <t>A.8.9</t>
+  </si>
+  <si>
+    <t>ISB-P14 Werkplekken, malware en kwetsbaarheden</t>
+  </si>
+  <si>
+    <t>A18</t>
+  </si>
+  <si>
+    <t>Een beleid voor back-ups en bewijs dat back-ups regelmatig worden getest.</t>
+  </si>
+  <si>
+    <t>A.8.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISB-P11 Back-up en herstel
+BEW-001 Bewijsregister periodieke controles</t>
+  </si>
+  <si>
+    <t>A19</t>
+  </si>
+  <si>
+    <t>Logbestanden van activiteiten en beveiligingsgebeurtenissen, bewaard en beschermd.</t>
+  </si>
+  <si>
+    <t>A.8.15</t>
+  </si>
+  <si>
+    <t>ISB-P10 Logging en monitoring</t>
+  </si>
+  <si>
+    <t>A20</t>
+  </si>
+  <si>
+    <t>Regels voor het gebruik van cryptografie, inclusief het beheer van sleutels.</t>
+  </si>
+  <si>
+    <t>A.8.24</t>
+  </si>
+  <si>
+    <t>ISB-P09 Versleuteling</t>
+  </si>
+  <si>
+    <t>A21</t>
+  </si>
+  <si>
+    <t>Vastgelegde uitgangspunten voor het ontwerpen van veilige systemen.</t>
+  </si>
+  <si>
+    <t>A.8.27</t>
+  </si>
+  <si>
+    <t>ISB-P13 Veilige softwareontwikkeling</t>
+  </si>
+  <si>
+    <t>A22</t>
+  </si>
+  <si>
+    <t>Procedures voor het beheren van wijzigingen in systemen.</t>
+  </si>
+  <si>
+    <t>A.8.32</t>
+  </si>
+  <si>
+    <t>ISB-P08 Wijzigingen in systemen en projecten</t>
   </si>
   <si>
     <t>Overzicht</t>
@@ -1343,7 +1531,7 @@
     <tabColor rgb="FFC2410C"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1815,18 +2003,18 @@
       <c r="G25" s="15"/>
       <c r="H25" s="17"/>
       <c r="I25" s="18" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B26" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="C26" s="16" t="s">
         <v>118</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>119</v>
       </c>
       <c r="D26" s="15"/>
       <c r="E26" s="15"/>
@@ -1834,18 +2022,322 @@
       <c r="G26" s="15"/>
       <c r="H26" s="17"/>
       <c r="I26" s="18" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
         <v>120</v>
       </c>
+      <c r="B27" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="18" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="18" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="18" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="18" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="18" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="18" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="18" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="18" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="17"/>
+      <c r="I37" s="18" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="17"/>
+      <c r="I38" s="18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="17"/>
+      <c r="I39" s="18" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="17"/>
+      <c r="I40" s="18" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="17"/>
+      <c r="I41" s="18" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="17"/>
+      <c r="I42" s="18" t="s">
+        <v>180</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:I26"/>
+  <autoFilter ref="A3:I42"/>
   <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A20:I20"/>
   </mergeCells>
-  <conditionalFormatting sqref="D5:D26">
+  <conditionalFormatting sqref="D5:D42">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("Voldoet",D5)))</formula>
     </cfRule>
@@ -1860,7 +2352,7 @@
     <dataValidation type="list" allowBlank="1" sqref="D10:D19">
       <formula1>"✓ Voldoet,! Deels,✕ Ontbreekt,– Niet van toepassing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D21:D26">
+    <dataValidation type="list" allowBlank="1" sqref="D21:D42">
       <formula1>"✓ Voldoet,! Deels,✕ Ontbreekt,– Niet van toepassing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D5:D19">
@@ -1890,38 +2382,38 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
-        <v>121</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>122</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
-        <v>123</v>
+        <v>183</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>124</v>
+        <v>184</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>125</v>
+        <v>185</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>126</v>
+        <v>186</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>127</v>
+        <v>187</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>128</v>
+        <v>188</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="H4" s="21" t="s">
-        <v>130</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1955,19 +2447,19 @@
         <v>97</v>
       </c>
       <c r="B6" s="23">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C6" s="23">
-        <f>COUNTIF(Checklist!D21:D26,"✓ Voldoet")</f>
+        <f>COUNTIF(Checklist!D21:D42,"✓ Voldoet")</f>
       </c>
       <c r="D6" s="23">
-        <f>COUNTIF(Checklist!D21:D26,"! Deels")</f>
+        <f>COUNTIF(Checklist!D21:D42,"! Deels")</f>
       </c>
       <c r="E6" s="23">
-        <f>COUNTIF(Checklist!D21:D26,"✕ Ontbreekt")</f>
+        <f>COUNTIF(Checklist!D21:D42,"✕ Ontbreekt")</f>
       </c>
       <c r="F6" s="23">
-        <f>COUNTIF(Checklist!D21:D26,"– Niet van toepassing")</f>
+        <f>COUNTIF(Checklist!D21:D42,"– Niet van toepassing")</f>
       </c>
       <c r="G6" s="23">
         <f>B6-C6-F6</f>
@@ -1978,7 +2470,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>131</v>
+        <v>191</v>
       </c>
       <c r="B7" s="26">
         <f>SUM(B5:B6)</f>
@@ -2016,7 +2508,7 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
-        <v>132</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2032,7 +2524,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{87AF0854-4ACF-42EF-B2FB-D0240023B57E}</x14:id>
+          <x14:id>{1AA2310A-0D65-4854-958A-3978F84614BA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -2046,7 +2538,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{87AF0854-4ACF-42EF-B2FB-D0240023B57E}">
+          <x14:cfRule type="dataBar" id="{1AA2310A-0D65-4854-958A-3978F84614BA}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>